<commit_message>
feat(application): require birth region in applications
</commit_message>
<xml_diff>
--- a/outputs/bulk-excel-templates-20260818/고등학교_학생증_단체신청_양식_v1.1.xlsx
+++ b/outputs/bulk-excel-templates-20260818/고등학교_학생증_단체신청_양식_v1.1.xlsx
@@ -327,7 +327,7 @@
     </comment>
     <comment ref="F3" authorId="0" shapeId="0">
       <text>
-        <t>선택 항목입니다. 자세한 형식과 예시는 작성안내 시트를 확인하세요.</t>
+        <t>필수 항목입니다. 자세한 형식과 예시는 작성안내 시트를 확인하세요.</t>
       </text>
     </comment>
     <comment ref="G3" authorId="0" shapeId="0">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>국적</t>
+          <t>출생국가</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -2977,16 +2977,15 @@
       <formula1>DATE(1900,1,1)</formula1>
       <formula2>TODAY()</formula2>
     </dataValidation>
-    <dataValidation sqref="D4:D103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="국적 입력 오류" error="목록의 ISO 2자리 대문자 국가코드를 선택하세요." promptTitle="국적 입력 오류" prompt="필수 항목입니다. 예: KR, US, JP" type="list" errorStyle="stop">
+    <dataValidation sqref="D4:D103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="출생국가 입력 오류" error="목록의 ISO 2자리 대문자 국가코드를 선택하세요." promptTitle="출생국가 입력 오류" prompt="필수 항목입니다. 예: KR, US, JP" type="list" errorStyle="stop">
       <formula1>CountryCodes</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="출생시간 입력 오류" error="HH:mm 또는 HH:mm:ss 형식으로 입력하세요." promptTitle="출생시간 입력 오류" prompt="선택 항목입니다. 예: 14:30" type="time" errorStyle="stop">
       <formula1>TIME(0,0,0)</formula1>
       <formula2>TIME(23,59,59)</formula2>
     </dataValidation>
-    <dataValidation sqref="F4:F103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="출생지역 입력 오류" error="출생지역은 최대 200자입니다." promptTitle="출생지역 입력 오류" prompt="선택 항목입니다." type="textLength" errorStyle="stop">
-      <formula1>0</formula1>
-      <formula2>200</formula2>
+    <dataValidation sqref="F4:F103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="출생지역 입력 오류" error="출생지역은 필수이며 태어난 도시명을 최대 200자로 입력해야 합니다." promptTitle="출생지역 입력 오류" prompt="태어난 도시명을 입력하세요. 예: Chicago, London, Tokyo, Beijing, Los Angeles" type="custom" errorStyle="stop">
+      <formula1>AND(F4&lt;&gt;"",LEN(TRIM(F4))&lt;=200)</formula1>
     </dataValidation>
     <dataValidation sqref="G4:G103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="성별 입력 오류" error="MALE 또는 FEMALE을 선택하세요." promptTitle="성별 입력 오류" prompt="필수 항목입니다." type="list" errorStyle="stop">
       <formula1>GenderCodes</formula1>
@@ -3191,7 +3190,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>국적 · 필수</t>
+          <t>출생국가 · 필수</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
@@ -3212,15 +3211,15 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>출생지역 · 선택</t>
+          <t>출생지역(출신지역) · 필수</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>최대 200자로 입력합니다.</t>
+          <t>태어난 도시명을 최대 200자로 입력합니다. 예: Chicago, London, Tokyo, Beijing, Los Angeles</t>
         </is>
       </c>
     </row>

</xml_diff>